<commit_message>
Update concatenator and uploader scripts
</commit_message>
<xml_diff>
--- a/templates/uploader_template.xlsx
+++ b/templates/uploader_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth_9lb83h2\Desktop\TONIK\Coding Projects\competitor-uploader\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth_9lb83h2\Desktop\TONIK\Coding Projects\competitor-uploader\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89AFB4BF-B53E-43FB-8333-AB2A3031FF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2F6FA22-FE62-4A63-BA74-880CF181CBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9870" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FEFC82FB-9138-4974-98A6-92D033F7767D}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="45">
   <si>
     <t>purpleKey</t>
   </si>
@@ -149,6 +149,12 @@
   </si>
   <si>
     <t>Stormtech Gaisano Mall Tabunok</t>
+  </si>
+  <si>
+    <t>billeaseSales</t>
+  </si>
+  <si>
+    <t>billeaseHeadcount</t>
   </si>
 </sst>
 </file>
@@ -1009,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{574A2230-ABBC-44FC-B807-DB87895D3D8E}">
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -1036,9 +1042,11 @@
     <col min="22" max="22" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1111,8 +1119,14 @@
       <c r="X1" t="s">
         <v>23</v>
       </c>
+      <c r="Y1" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>24</v>
       </c>
@@ -1171,7 +1185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>31</v>
       </c>
@@ -1230,7 +1244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>32</v>
       </c>
@@ -1289,7 +1303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>33</v>
       </c>
@@ -1348,7 +1362,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -1407,7 +1421,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>37</v>
       </c>
@@ -1466,7 +1480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>39</v>
       </c>
@@ -1525,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>40</v>
       </c>
@@ -1584,7 +1598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>41</v>
       </c>
@@ -1643,7 +1657,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>42</v>
       </c>

</xml_diff>

<commit_message>
Add billeaseSales/billeaseHeadcount columns, upload_timestamp, and Mac credentials path
- Added billeaseSales and billeaseHeadcount fields to schema and templates
- Concatenator now stamps upload_timestamp on each row at run time
- Uploader uses Manila TZ timestamp, flexible multi-format date parser, and load_table_from_dataframe
- Updated .gitignore to exclude adc.json, .venv_runner/, data/, and log files
- Added MACOS_SETUP.txt, run scripts, and sample_run.txt
- Updated GOOGLE_APPLICATION_CREDENTIALS to local Mac path

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/uploader_template.xlsx
+++ b/templates/uploader_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\matth_9lb83h2\Desktop\TONIK\Coding Projects\competitor-uploader\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewfranzoco/Desktop/Projects/competitor-uploader/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2F6FA22-FE62-4A63-BA74-880CF181CBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C2EE469-7B0C-7840-8581-487D711BBF67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9870" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FEFC82FB-9138-4974-98A6-92D033F7767D}"/>
+    <workbookView xWindow="0" yWindow="860" windowWidth="34200" windowHeight="19560" xr2:uid="{FEFC82FB-9138-4974-98A6-92D033F7767D}"/>
   </bookViews>
   <sheets>
     <sheet name="uploader_template" sheetId="1" r:id="rId1"/>
@@ -151,10 +151,10 @@
     <t>Stormtech Gaisano Mall Tabunok</t>
   </si>
   <si>
+    <t>billeaseHeadcount</t>
+  </si>
+  <si>
     <t>billeaseSales</t>
-  </si>
-  <si>
-    <t>billeaseHeadcount</t>
   </si>
 </sst>
 </file>
@@ -1016,37 +1016,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{574A2230-ABBC-44FC-B807-DB87895D3D8E}">
   <dimension ref="A1:Z11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="17" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5" customWidth="1"/>
+    <col min="16" max="16" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.5" customWidth="1"/>
+    <col min="26" max="26" width="15.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1090,43 +1090,43 @@
         <v>13</v>
       </c>
       <c r="O1" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>22</v>
-      </c>
-      <c r="X1" t="s">
-        <v>23</v>
       </c>
       <c r="Y1" t="s">
         <v>43</v>
       </c>
       <c r="Z1" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>24</v>
       </c>
@@ -1157,24 +1157,21 @@
       <c r="M2">
         <v>4549</v>
       </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
       <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
         <v>26297</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>664362</v>
       </c>
-      <c r="R2">
+      <c r="S2">
         <v>30497</v>
       </c>
-      <c r="S2">
+      <c r="T2">
         <v>195794</v>
       </c>
-      <c r="T2">
-        <v>1</v>
-      </c>
       <c r="U2">
         <v>1</v>
       </c>
@@ -1184,8 +1181,11 @@
       <c r="W2">
         <v>1</v>
       </c>
+      <c r="X2">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>31</v>
       </c>
@@ -1216,35 +1216,35 @@
       <c r="M3">
         <v>88890</v>
       </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
       <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
         <v>87500</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>280765</v>
       </c>
-      <c r="R3">
+      <c r="S3">
         <v>114511</v>
       </c>
-      <c r="S3">
+      <c r="T3">
         <v>143674</v>
       </c>
-      <c r="T3">
+      <c r="U3">
         <v>0.5</v>
       </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
       <c r="V3">
         <v>0</v>
       </c>
       <c r="W3">
         <v>0</v>
       </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>32</v>
       </c>
@@ -1275,24 +1275,21 @@
       <c r="M4">
         <v>0</v>
       </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
       <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
         <v>24990</v>
       </c>
-      <c r="Q4">
+      <c r="R4">
         <v>278020</v>
       </c>
-      <c r="R4">
+      <c r="S4">
         <v>86990</v>
       </c>
-      <c r="S4">
+      <c r="T4">
         <v>360000</v>
       </c>
-      <c r="T4">
-        <v>1</v>
-      </c>
       <c r="U4">
         <v>1</v>
       </c>
@@ -1302,8 +1299,11 @@
       <c r="W4">
         <v>1</v>
       </c>
+      <c r="X4">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>33</v>
       </c>
@@ -1334,35 +1334,35 @@
       <c r="M5">
         <v>15596</v>
       </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
       <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
         <v>155809</v>
       </c>
-      <c r="Q5">
+      <c r="R5">
         <v>943300</v>
       </c>
-      <c r="R5">
+      <c r="S5">
         <v>133434</v>
       </c>
-      <c r="S5">
+      <c r="T5">
         <v>295752</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <v>0.5</v>
       </c>
-      <c r="U5">
-        <v>1</v>
-      </c>
       <c r="V5">
         <v>1</v>
       </c>
       <c r="W5">
         <v>1</v>
       </c>
+      <c r="X5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>34</v>
       </c>
@@ -1393,23 +1393,20 @@
       <c r="M6">
         <v>0</v>
       </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
       <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
         <v>10000000</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>5000000</v>
       </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
       <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
         <v>2000000</v>
-      </c>
-      <c r="T6">
-        <v>3</v>
       </c>
       <c r="U6">
         <v>3</v>
@@ -1420,8 +1417,11 @@
       <c r="W6">
         <v>3</v>
       </c>
+      <c r="X6">
+        <v>3</v>
+      </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>37</v>
       </c>
@@ -1452,26 +1452,23 @@
       <c r="M7">
         <v>50000</v>
       </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
       <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
         <v>200000</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>710083</v>
       </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
       <c r="S7">
         <v>0</v>
       </c>
       <c r="T7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7">
         <v>0</v>
@@ -1479,8 +1476,11 @@
       <c r="W7">
         <v>0</v>
       </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B8" t="s">
         <v>39</v>
       </c>
@@ -1511,24 +1511,21 @@
       <c r="M8">
         <v>14399</v>
       </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
       <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
         <v>109600</v>
       </c>
-      <c r="Q8">
+      <c r="R8">
         <v>688965</v>
       </c>
-      <c r="R8">
+      <c r="S8">
         <v>174400</v>
       </c>
-      <c r="S8">
+      <c r="T8">
         <v>375913</v>
       </c>
-      <c r="T8">
-        <v>1</v>
-      </c>
       <c r="U8">
         <v>1</v>
       </c>
@@ -1538,8 +1535,11 @@
       <c r="W8">
         <v>1</v>
       </c>
+      <c r="X8">
+        <v>1</v>
+      </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B9" t="s">
         <v>40</v>
       </c>
@@ -1570,24 +1570,21 @@
       <c r="M9">
         <v>0</v>
       </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
       <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
         <v>234508</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>322655</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>12990</v>
       </c>
-      <c r="S9">
+      <c r="T9">
         <v>21897</v>
       </c>
-      <c r="T9">
-        <v>1</v>
-      </c>
       <c r="U9">
         <v>1</v>
       </c>
@@ -1597,8 +1594,11 @@
       <c r="W9">
         <v>1</v>
       </c>
+      <c r="X9">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
         <v>41</v>
       </c>
@@ -1629,24 +1629,21 @@
       <c r="M10">
         <v>0</v>
       </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
       <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
         <v>191518</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>968487</v>
       </c>
-      <c r="R10">
+      <c r="S10">
         <v>308613</v>
       </c>
-      <c r="S10">
+      <c r="T10">
         <v>164090</v>
       </c>
-      <c r="T10">
-        <v>1</v>
-      </c>
       <c r="U10">
         <v>1</v>
       </c>
@@ -1656,8 +1653,11 @@
       <c r="W10">
         <v>1</v>
       </c>
+      <c r="X10">
+        <v>1</v>
+      </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
       <c r="B11" t="s">
         <v>42</v>
       </c>
@@ -1688,24 +1688,21 @@
       <c r="M11">
         <v>58896</v>
       </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
       <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
         <v>129140</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>653356</v>
       </c>
-      <c r="R11">
+      <c r="S11">
         <v>204492</v>
       </c>
-      <c r="S11">
+      <c r="T11">
         <v>287386</v>
       </c>
-      <c r="T11">
-        <v>1</v>
-      </c>
       <c r="U11">
         <v>1</v>
       </c>
@@ -1713,6 +1710,9 @@
         <v>1</v>
       </c>
       <c r="W11">
+        <v>1</v>
+      </c>
+      <c r="X11">
         <v>1</v>
       </c>
     </row>

</xml_diff>